<commit_message>
Add 'Negative tests' to checklist. Refine 'Happy path'
</commit_message>
<xml_diff>
--- a/docs/checklists/checklist.xlsx
+++ b/docs/checklists/checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Practice\POSTMAN\docs\checklists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9A8398-2BE8-4844-99AC-1CDE3DF7BD79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DCE8945-AF2D-42B5-BE83-C756A09F133E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,14 +28,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="105">
   <si>
     <t>Happy Path (CRUD)</t>
   </si>
   <si>
-    <t>CHECKLIST FOR  RESTFful BOOKING API</t>
-  </si>
-  <si>
     <t>Ping</t>
   </si>
   <si>
@@ -69,9 +66,6 @@
     <t>PATCH</t>
   </si>
   <si>
-    <t>DEL</t>
-  </si>
-  <si>
     <t>Id</t>
   </si>
   <si>
@@ -274,13 +268,100 @@
   </si>
   <si>
     <t>"totalprice":1.5e2,</t>
+  </si>
+  <si>
+    <t>CHECKLIST FOR  RESTful BOOKING API</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>Expected Status Code</t>
+  </si>
+  <si>
+    <t>Actual Status</t>
+  </si>
+  <si>
+    <t>Endpoint URL</t>
+  </si>
+  <si>
+    <t>https://restful-booker.herokuapp.com/ping</t>
+  </si>
+  <si>
+    <t>https://restful-booker.herokuapp.com/auth</t>
+  </si>
+  <si>
+    <t>https://restful-booker.herokuapp.com/booking</t>
+  </si>
+  <si>
+    <t>https://restful-booker.herokuapp.com/booking/{{bookingId}}</t>
+  </si>
+  <si>
+    <t>Negative Tests</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>Create Booking - Additional field</t>
+  </si>
+  <si>
+    <t>{
+    "firstname" : "Jim",
+    "lastname" : "Brown",
+    "totalprice" : 123,
+    "depositpaid" : true,
+    "oneMoreField": "veryUsefulInfo",
+    "bookingdates" : {
+        "checkin" : "2018-01-01",
+        "checkout" : "2019-01-01"
+    },
+    "additionalneeds" : "Breakfast"
+}</t>
+  </si>
+  <si>
+    <t>Server accepts this request, but returns standard body without any additional fields</t>
+  </si>
+  <si>
+    <t>Patch w/o token</t>
+  </si>
+  <si>
+    <t>Update w/o token</t>
+  </si>
+  <si>
+    <t>Create w/o token</t>
+  </si>
+  <si>
+    <t>*standard body with valid payload*</t>
+  </si>
+  <si>
+    <t>{ "username": "admin" }</t>
+  </si>
+  <si>
+    <t>Server accepts this request, returns 200 OK, with message - "Bad credentials"</t>
+  </si>
+  <si>
+    <t>Get token - w/o password</t>
+  </si>
+  <si>
+    <t>Get token - w/o username</t>
+  </si>
+  <si>
+    <t>{ "password" : "password123" }</t>
+  </si>
+  <si>
+    <t>Get token - non-existent user</t>
+  </si>
+  <si>
+    <t>{    "username" : "admin123",
+    "password" : "password123"}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -322,19 +403,21 @@
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -349,7 +432,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="44">
     <border>
       <left/>
       <right/>
@@ -431,19 +514,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -663,17 +733,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -775,40 +834,193 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -820,10 +1032,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -832,17 +1044,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -851,88 +1063,177 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1216,171 +1517,238 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X38"/>
+  <dimension ref="A1:X53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.88671875" customWidth="1"/>
     <col min="3" max="3" width="21" style="2" customWidth="1"/>
-    <col min="6" max="6" width="22.33203125" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.21875" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="47" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="48"/>
+      <c r="R1" s="48"/>
+      <c r="S1" s="48"/>
+      <c r="T1" s="48"/>
+      <c r="U1" s="48"/>
+      <c r="V1" s="48"/>
+      <c r="W1" s="48"/>
+      <c r="X1" s="49"/>
+    </row>
+    <row r="2" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="68" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="69"/>
+      <c r="T2" s="69"/>
+      <c r="U2" s="69"/>
+      <c r="V2" s="69"/>
+      <c r="W2" s="69"/>
+      <c r="X2" s="70"/>
+    </row>
+    <row r="3" spans="1:24" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="63" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="64" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="65" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="66" t="s">
+        <v>82</v>
+      </c>
+      <c r="F3" s="67" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="59"/>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A4" s="6">
         <v>1</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="44"/>
-      <c r="V1" s="44"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="45"/>
-    </row>
-    <row r="2" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="46" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="48"/>
-      <c r="O2" s="48"/>
-      <c r="P2" s="48"/>
-      <c r="Q2" s="48"/>
-      <c r="R2" s="48"/>
-      <c r="S2" s="48"/>
-      <c r="T2" s="48"/>
-      <c r="U2" s="48"/>
-      <c r="V2" s="48"/>
-      <c r="W2" s="48"/>
-      <c r="X2" s="49"/>
-    </row>
-    <row r="3" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A4" s="7">
+      <c r="B4" s="77" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="D4" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="71">
+        <v>201</v>
+      </c>
+      <c r="F4" s="72">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="B5" s="78" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="10"/>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" s="11">
-        <v>2</v>
-      </c>
-      <c r="B5" s="12" t="s">
+      <c r="E5" s="24">
+        <v>200</v>
+      </c>
+      <c r="F5" s="73">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A6" s="8">
         <v>3</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="B6" s="79" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="24">
+        <v>200</v>
+      </c>
+      <c r="F6" s="73">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A7" s="8">
+        <v>4</v>
+      </c>
+      <c r="B7" s="80" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="14"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6" s="11">
-        <v>3</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="14"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A7" s="11">
-        <v>4</v>
-      </c>
-      <c r="B7" s="12" t="s">
+      <c r="E7" s="24">
+        <v>200</v>
+      </c>
+      <c r="F7" s="73">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A8" s="8">
         <v>5</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="B8" s="79" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="14"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A8" s="11">
-        <v>5</v>
-      </c>
-      <c r="B8" s="12" t="s">
+      <c r="E8" s="24">
+        <v>200</v>
+      </c>
+      <c r="F8" s="73">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A9" s="8">
         <v>6</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="14"/>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="11">
+      <c r="B9" s="78" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="D9" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="24">
+        <v>201</v>
+      </c>
+      <c r="F9" s="73">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="10">
         <v>7</v>
       </c>
-      <c r="C9" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="14"/>
-    </row>
-    <row r="10" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="15">
+      <c r="B10" s="81" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="D10" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="18"/>
+      <c r="E10" s="74">
+        <v>404</v>
+      </c>
+      <c r="F10" s="75">
+        <v>404</v>
+      </c>
     </row>
     <row r="11" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A11" s="50" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" s="51"/>
       <c r="C11" s="51"/>
@@ -1406,20 +1774,22 @@
       <c r="W11" s="51"/>
       <c r="X11" s="52"/>
     </row>
-    <row r="12" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:24" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>17</v>
+      <c r="B12" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="58" t="s">
+        <v>82</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -1442,21 +1812,21 @@
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="31">
+        <v>17</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="22">
         <v>200</v>
       </c>
-      <c r="E13" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="35"/>
+      <c r="E13" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="26"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -1478,20 +1848,20 @@
     </row>
     <row r="14" spans="1:24" ht="28.2" x14ac:dyDescent="0.3">
       <c r="A14" s="54"/>
-      <c r="B14" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" s="32">
+      <c r="B14" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="23">
         <v>400</v>
       </c>
-      <c r="E14" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="36" t="s">
-        <v>43</v>
+      <c r="E14" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="27" t="s">
+        <v>41</v>
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
@@ -1514,20 +1884,20 @@
     </row>
     <row r="15" spans="1:24" ht="28.2" x14ac:dyDescent="0.3">
       <c r="A15" s="54"/>
-      <c r="B15" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="32">
+      <c r="B15" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="23">
         <v>400</v>
       </c>
-      <c r="E15" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="F15" s="36" t="s">
-        <v>43</v>
+      <c r="E15" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="27" t="s">
+        <v>41</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -1550,20 +1920,20 @@
     </row>
     <row r="16" spans="1:24" ht="42" x14ac:dyDescent="0.3">
       <c r="A16" s="54"/>
-      <c r="B16" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" s="32">
+      <c r="B16" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="23">
         <v>400</v>
       </c>
-      <c r="E16" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="F16" s="36" t="s">
-        <v>46</v>
+      <c r="E16" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="27" t="s">
+        <v>44</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -1586,20 +1956,20 @@
     </row>
     <row r="17" spans="1:24" ht="42" x14ac:dyDescent="0.3">
       <c r="A17" s="54"/>
-      <c r="B17" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C17" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="32">
+      <c r="B17" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="23">
         <v>400</v>
       </c>
-      <c r="E17" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="F17" s="36" t="s">
-        <v>45</v>
+      <c r="E17" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="27" t="s">
+        <v>43</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
@@ -1622,79 +1992,79 @@
     </row>
     <row r="18" spans="1:24" ht="42" x14ac:dyDescent="0.3">
       <c r="A18" s="54"/>
-      <c r="B18" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="33">
+      <c r="B18" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" s="24">
         <v>400</v>
       </c>
-      <c r="E18" s="34" t="s">
+      <c r="E18" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F18" s="27" t="s">
         <v>42</v>
-      </c>
-      <c r="F18" s="36" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:24" ht="28.2" x14ac:dyDescent="0.3">
       <c r="A19" s="54"/>
-      <c r="B19" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" s="33">
+      <c r="B19" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="24">
         <v>400</v>
       </c>
-      <c r="E19" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="F19" s="36" t="s">
-        <v>43</v>
+      <c r="E19" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="27" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:24" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="54"/>
-      <c r="B20" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="D20" s="33">
+      <c r="B20" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" s="24">
         <v>400</v>
       </c>
-      <c r="E20" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="F20" s="37" t="s">
-        <v>47</v>
+      <c r="E20" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="28" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:24" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="55"/>
-      <c r="B21" s="38" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" s="39" t="s">
-        <v>39</v>
-      </c>
-      <c r="D21" s="40">
+      <c r="B21" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="31">
         <v>400</v>
       </c>
-      <c r="E21" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F21" s="42" t="s">
-        <v>43</v>
+      <c r="E21" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="33" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="56" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B22" s="57"/>
       <c r="C22" s="57"/>
@@ -1722,18 +2092,20 @@
     </row>
     <row r="23" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="63" t="s">
-        <v>24</v>
-      </c>
-      <c r="D23" s="64" t="s">
-        <v>21</v>
-      </c>
-      <c r="E23" s="65" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>41</v>
+      <c r="B23" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
@@ -1755,22 +2127,22 @@
       <c r="X23" s="1"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A24" s="62" t="s">
-        <v>19</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="D24" s="31">
+      <c r="A24" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="22">
         <v>200</v>
       </c>
-      <c r="E24" s="30" t="s">
-        <v>40</v>
-      </c>
-      <c r="F24" s="35"/>
+      <c r="E24" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24" s="26"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
@@ -1790,22 +2162,22 @@
       <c r="W24" s="1"/>
       <c r="X24" s="1"/>
     </row>
-    <row r="25" spans="1:24" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="60"/>
-      <c r="B25" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="D25" s="32">
+    <row r="25" spans="1:24" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="45"/>
+      <c r="B25" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D25" s="23">
         <v>400</v>
       </c>
-      <c r="E25" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F25" s="36" t="s">
-        <v>63</v>
+      <c r="E25" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" s="27" t="s">
+        <v>61</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
@@ -1826,22 +2198,22 @@
       <c r="W25" s="1"/>
       <c r="X25" s="1"/>
     </row>
-    <row r="26" spans="1:24" ht="56.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="60"/>
-      <c r="B26" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C26" s="27" t="s">
-        <v>64</v>
-      </c>
-      <c r="D26" s="32">
+    <row r="26" spans="1:24" ht="42" x14ac:dyDescent="0.3">
+      <c r="A26" s="45"/>
+      <c r="B26" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" s="23">
         <v>400</v>
       </c>
-      <c r="E26" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F26" s="36" t="s">
-        <v>65</v>
+      <c r="E26" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26" s="27" t="s">
+        <v>63</v>
       </c>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
@@ -1862,22 +2234,22 @@
       <c r="W26" s="1"/>
       <c r="X26" s="1"/>
     </row>
-    <row r="27" spans="1:24" ht="56.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="60"/>
-      <c r="B27" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C27" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="32">
+    <row r="27" spans="1:24" ht="42" x14ac:dyDescent="0.3">
+      <c r="A27" s="45"/>
+      <c r="B27" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" s="23">
         <v>400</v>
       </c>
-      <c r="E27" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F27" s="36" t="s">
-        <v>65</v>
+      <c r="E27" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="27" t="s">
+        <v>63</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
@@ -1898,22 +2270,22 @@
       <c r="W27" s="1"/>
       <c r="X27" s="1"/>
     </row>
-    <row r="28" spans="1:24" ht="70.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="60"/>
-      <c r="B28" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" s="66" t="s">
-        <v>67</v>
-      </c>
-      <c r="D28" s="32">
+    <row r="28" spans="1:24" ht="69.599999999999994" x14ac:dyDescent="0.3">
+      <c r="A28" s="45"/>
+      <c r="B28" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="37" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" s="23">
         <v>400</v>
       </c>
-      <c r="E28" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F28" s="36" t="s">
-        <v>68</v>
+      <c r="E28" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F28" s="27" t="s">
+        <v>66</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
@@ -1934,172 +2306,452 @@
       <c r="W28" s="1"/>
       <c r="X28" s="1"/>
     </row>
-    <row r="29" spans="1:24" ht="56.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="60"/>
-      <c r="B29" s="22" t="s">
+    <row r="29" spans="1:24" ht="42" x14ac:dyDescent="0.3">
+      <c r="A29" s="45"/>
+      <c r="B29" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="D29" s="23">
+        <v>400</v>
+      </c>
+      <c r="E29" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" ht="55.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="45"/>
+      <c r="B30" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D30" s="23">
+        <v>400</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A31" s="45"/>
+      <c r="B31" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="66" t="s">
-        <v>69</v>
-      </c>
-      <c r="D29" s="32">
+      <c r="C31" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" s="23">
+        <v>200</v>
+      </c>
+      <c r="E31" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F31" s="27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A32" s="45"/>
+      <c r="B32" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="D32" s="23">
+        <v>200</v>
+      </c>
+      <c r="E32" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F32" s="27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" ht="55.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="45"/>
+      <c r="B33" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D33" s="23">
         <v>400</v>
       </c>
-      <c r="E29" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F29" s="36" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:24" ht="56.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="60"/>
-      <c r="B30" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="C30" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="D30" s="32">
+      <c r="E33" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F33" s="27" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A34" s="45"/>
+      <c r="B34" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D34" s="23">
+        <v>200</v>
+      </c>
+      <c r="E34" s="84" t="s">
+        <v>38</v>
+      </c>
+      <c r="F34" s="38"/>
+    </row>
+    <row r="35" spans="1:24" ht="69" x14ac:dyDescent="0.3">
+      <c r="A35" s="45"/>
+      <c r="B35" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C35" s="39" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35" s="23">
         <v>400</v>
       </c>
-      <c r="E30" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F30" s="36" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="31" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="60"/>
-      <c r="B31" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="C31" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="D31" s="32">
+      <c r="E35" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F35" s="27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A36" s="45"/>
+      <c r="B36" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" s="23">
         <v>200</v>
       </c>
-      <c r="E31" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F31" s="36" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="32" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="60"/>
-      <c r="B32" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="C32" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="D32" s="32">
+      <c r="E36" s="84" t="s">
+        <v>38</v>
+      </c>
+      <c r="F36" s="38"/>
+    </row>
+    <row r="37" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="46"/>
+      <c r="B37" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="C37" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" s="41">
         <v>200</v>
       </c>
-      <c r="E32" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F32" s="36" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="56.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="60"/>
-      <c r="B33" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33" s="28" t="s">
-        <v>75</v>
-      </c>
-      <c r="D33" s="32">
-        <v>400</v>
-      </c>
-      <c r="E33" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F33" s="36" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="60"/>
-      <c r="B34" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="C34" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="D34" s="32">
+      <c r="E37" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="F37" s="43"/>
+    </row>
+    <row r="38" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A38" s="56" t="s">
+        <v>89</v>
+      </c>
+      <c r="B38" s="57"/>
+      <c r="C38" s="57"/>
+      <c r="D38" s="57"/>
+      <c r="E38" s="57"/>
+      <c r="F38" s="57"/>
+      <c r="G38" s="57"/>
+      <c r="H38" s="57"/>
+      <c r="I38" s="51"/>
+      <c r="J38" s="51"/>
+      <c r="K38" s="51"/>
+      <c r="L38" s="51"/>
+      <c r="M38" s="51"/>
+      <c r="N38" s="51"/>
+      <c r="O38" s="51"/>
+      <c r="P38" s="51"/>
+      <c r="Q38" s="51"/>
+      <c r="R38" s="51"/>
+      <c r="S38" s="51"/>
+      <c r="T38" s="51"/>
+      <c r="U38" s="51"/>
+      <c r="V38" s="51"/>
+      <c r="W38" s="51"/>
+      <c r="X38" s="52"/>
+    </row>
+    <row r="39" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="3"/>
+      <c r="B39" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" s="91" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="92" t="s">
+        <v>90</v>
+      </c>
+      <c r="E39" s="85" t="s">
+        <v>22</v>
+      </c>
+      <c r="F39" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="B40" s="98" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" s="96" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="99" t="s">
+        <v>87</v>
+      </c>
+      <c r="E40" s="100" t="s">
+        <v>92</v>
+      </c>
+      <c r="F40" s="101">
         <v>200</v>
       </c>
-      <c r="E34" s="30" t="s">
+      <c r="G40" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="H40" s="103" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A41" s="45"/>
+      <c r="B41" s="104" t="s">
+        <v>96</v>
+      </c>
+      <c r="C41" s="90" t="s">
+        <v>9</v>
+      </c>
+      <c r="D41" s="95" t="s">
+        <v>88</v>
+      </c>
+      <c r="E41" s="86" t="s">
+        <v>97</v>
+      </c>
+      <c r="F41" s="23">
+        <v>403</v>
+      </c>
+      <c r="G41" s="84" t="s">
+        <v>38</v>
+      </c>
+      <c r="H41" s="27"/>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A42" s="45"/>
+      <c r="B42" s="104" t="s">
+        <v>95</v>
+      </c>
+      <c r="C42" s="90" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" s="95" t="s">
+        <v>88</v>
+      </c>
+      <c r="E42" s="86" t="s">
+        <v>97</v>
+      </c>
+      <c r="F42" s="23">
+        <v>403</v>
+      </c>
+      <c r="G42" s="84" t="s">
+        <v>38</v>
+      </c>
+      <c r="H42" s="27"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A43" s="45"/>
+      <c r="B43" s="104" t="s">
+        <v>94</v>
+      </c>
+      <c r="C43" s="90" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="95" t="s">
+        <v>88</v>
+      </c>
+      <c r="E43" s="86" t="s">
+        <v>97</v>
+      </c>
+      <c r="F43" s="23">
+        <v>403</v>
+      </c>
+      <c r="G43" s="84" t="s">
+        <v>38</v>
+      </c>
+      <c r="H43" s="27"/>
+    </row>
+    <row r="44" spans="1:24" ht="42" x14ac:dyDescent="0.3">
+      <c r="A44" s="45"/>
+      <c r="B44" s="105" t="s">
+        <v>103</v>
+      </c>
+      <c r="C44" s="90" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="97" t="s">
+        <v>86</v>
+      </c>
+      <c r="E44" s="109" t="s">
+        <v>104</v>
+      </c>
+      <c r="F44" s="108">
+        <v>401</v>
+      </c>
+      <c r="G44" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="F34" s="67"/>
-    </row>
-    <row r="35" spans="1:6" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="60"/>
-      <c r="B35" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="C35" s="68" t="s">
-        <v>77</v>
-      </c>
-      <c r="D35" s="32">
-        <v>400</v>
-      </c>
-      <c r="E35" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="F35" s="36" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="60"/>
-      <c r="B36" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C36" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="D36" s="32">
-        <v>200</v>
-      </c>
-      <c r="E36" s="30" t="s">
+      <c r="H44" s="27" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="45" spans="1:24" ht="42" x14ac:dyDescent="0.3">
+      <c r="A45" s="45"/>
+      <c r="B45" s="106" t="s">
+        <v>100</v>
+      </c>
+      <c r="C45" s="90" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" s="97" t="s">
+        <v>86</v>
+      </c>
+      <c r="E45" s="88" t="s">
+        <v>98</v>
+      </c>
+      <c r="F45" s="23">
+        <v>401</v>
+      </c>
+      <c r="G45" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="F36" s="67"/>
-    </row>
-    <row r="37" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="61"/>
-      <c r="B37" s="69" t="s">
-        <v>60</v>
-      </c>
-      <c r="C37" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="D37" s="70">
-        <v>200</v>
-      </c>
-      <c r="E37" s="71" t="s">
+      <c r="H45" s="27" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="46" spans="1:24" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A46" s="45"/>
+      <c r="B46" s="106" t="s">
+        <v>101</v>
+      </c>
+      <c r="C46" s="90" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" s="97" t="s">
+        <v>86</v>
+      </c>
+      <c r="E46" s="88" t="s">
+        <v>102</v>
+      </c>
+      <c r="F46" s="23">
+        <v>401</v>
+      </c>
+      <c r="G46" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="F37" s="72"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="58"/>
-      <c r="B38" s="58"/>
-      <c r="C38" s="59"/>
-      <c r="D38" s="58"/>
-      <c r="E38" s="58"/>
-      <c r="F38" s="58"/>
+      <c r="H46" s="27" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A47" s="45"/>
+      <c r="B47" s="104"/>
+      <c r="C47" s="90"/>
+      <c r="D47" s="60"/>
+      <c r="E47" s="87"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="83"/>
+      <c r="H47" s="27"/>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A48" s="45"/>
+      <c r="B48" s="106"/>
+      <c r="C48" s="90"/>
+      <c r="D48" s="60"/>
+      <c r="E48" s="87"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="83"/>
+      <c r="H48" s="27"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A49" s="45"/>
+      <c r="B49" s="104"/>
+      <c r="C49" s="90"/>
+      <c r="D49" s="60"/>
+      <c r="E49" s="87"/>
+      <c r="F49" s="23"/>
+      <c r="G49" s="83"/>
+      <c r="H49" s="27"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50" s="45"/>
+      <c r="B50" s="106"/>
+      <c r="C50" s="90"/>
+      <c r="D50" s="60"/>
+      <c r="E50" s="87"/>
+      <c r="F50" s="23"/>
+      <c r="G50" s="83"/>
+      <c r="H50" s="38"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A51" s="45"/>
+      <c r="B51" s="104"/>
+      <c r="C51" s="90"/>
+      <c r="D51" s="60"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="23"/>
+      <c r="G51" s="83"/>
+      <c r="H51" s="27"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A52" s="45"/>
+      <c r="B52" s="106"/>
+      <c r="C52" s="90"/>
+      <c r="D52" s="60"/>
+      <c r="E52" s="87"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="83"/>
+      <c r="H52" s="38"/>
+    </row>
+    <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="46"/>
+      <c r="B53" s="107"/>
+      <c r="C53" s="93"/>
+      <c r="D53" s="94"/>
+      <c r="E53" s="89"/>
+      <c r="F53" s="41"/>
+      <c r="G53" s="82"/>
+      <c r="H53" s="43"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="A38:X38"/>
+    <mergeCell ref="A40:A53"/>
     <mergeCell ref="A24:A37"/>
     <mergeCell ref="A1:X1"/>
     <mergeCell ref="A2:X2"/>
@@ -2107,8 +2759,11 @@
     <mergeCell ref="A13:A21"/>
     <mergeCell ref="A22:X22"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B7" r:id="rId1" xr:uid="{9A88E16A-6488-4038-BE51-669306FE468A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
   <ignoredErrors>
     <ignoredError sqref="C19" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Add E2E scenarios to checklist: 'Search by name', 'State persistence', 'Security'
</commit_message>
<xml_diff>
--- a/docs/checklists/checklist.xlsx
+++ b/docs/checklists/checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Practice\POSTMAN\docs\checklists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DCE8945-AF2D-42B5-BE83-C756A09F133E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02E3CFB4-B8CD-4C37-BE64-B1584B99242E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="128">
   <si>
     <t>Happy Path (CRUD)</t>
   </si>
@@ -356,12 +356,110 @@
     <t>{    "username" : "admin123",
     "password" : "password123"}</t>
   </si>
+  <si>
+    <t>E2E - Search by name</t>
+  </si>
+  <si>
+    <t>Get booking by name</t>
+  </si>
+  <si>
+    <t>Partial update</t>
+  </si>
+  <si>
+    <t>https://restful-booker.herokuapp.com/booking?firstname={{name}}</t>
+  </si>
+  <si>
+    <t>{
+    "username" : "admin",
+    "password" : "password123"
+}</t>
+  </si>
+  <si>
+    <t>*no payload*</t>
+  </si>
+  <si>
+    <t>{
+    "additionalneeds" : "Late checkout"
+}</t>
+  </si>
+  <si>
+    <t>All tests were completed via URL: "https://restful-booker.herokuapp.com/booking/{{bookingId}}" in the next order: POST, PUT, PATCH</t>
+  </si>
+  <si>
+    <t>STANDARD BODY WITH VALID PAYLOAD</t>
+  </si>
+  <si>
+    <t>{
+    "firstname" : "QA_TU123",
+    "lastname" : "SomeLastName",
+    "totalprice" : 111,
+    "depositpaid" : true,
+    "bookingdates" : {
+        "checkin" : "2026-03-15",
+        "checkout" : "2026-03-20"
+    },
+    "additionalneeds" : "Breakfast"
+}</t>
+  </si>
+  <si>
+    <t>E2E - State persistence</t>
+  </si>
+  <si>
+    <t>Get booking</t>
+  </si>
+  <si>
+    <t>{
+    "totalprice" : 222
+}</t>
+  </si>
+  <si>
+    <t>E2E - Security</t>
+  </si>
+  <si>
+    <t>Try to update booking</t>
+  </si>
+  <si>
+    <t>Try to partial update</t>
+  </si>
+  <si>
+    <t>Try to delete booking</t>
+  </si>
+  <si>
+    <t>Get non-mutated booking</t>
+  </si>
+  <si>
+    <t>{
+    "firstname" : "Name1",
+    "lastname" : "Lastname1",
+    "totalprice" : 222,
+    "depositpaid" : false,
+    "bookingdates" : {
+        "checkin" : "2026-03-30",
+        "checkout" : "2026-04-15"
+    },
+    "additionalneeds" : "Lunch"
+}</t>
+  </si>
+  <si>
+    <t>{
+    "totalprice" : 333
+}</t>
+  </si>
+  <si>
+    <t>End-to-end scenario to verify data integrity and state persistence after partial resource mutations using the PATCH method</t>
+  </si>
+  <si>
+    <t>End-to-end scenario to verify possibility for user to search booking by user's name and modify it via PATCH method</t>
+  </si>
+  <si>
+    <t>End-to-end scenario to verify that state-changing operations (PUT, PATCH, DELETE) are properly restricted to authorized users only</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -411,6 +509,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -432,7 +545,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="44">
+  <borders count="51">
     <border>
       <left/>
       <right/>
@@ -823,21 +936,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top/>
       <bottom style="thin">
@@ -993,6 +1091,98 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1000,7 +1190,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="155">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1087,48 +1277,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1136,24 +1284,15 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1166,17 +1305,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="34" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1204,33 +1343,175 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="41" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -1517,7 +1798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X53"/>
+  <dimension ref="A1:AD79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.88671875" customWidth="1"/>
@@ -1529,88 +1810,104 @@
     <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:30" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="97" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="48"/>
-      <c r="Q1" s="48"/>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="48"/>
-      <c r="U1" s="48"/>
-      <c r="V1" s="48"/>
-      <c r="W1" s="48"/>
-      <c r="X1" s="49"/>
-    </row>
-    <row r="2" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="68" t="s">
+      <c r="B1" s="98"/>
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98"/>
+      <c r="H1" s="98"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="98"/>
+      <c r="K1" s="98"/>
+      <c r="L1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="98"/>
+      <c r="O1" s="98"/>
+      <c r="P1" s="98"/>
+      <c r="Q1" s="98"/>
+      <c r="R1" s="98"/>
+      <c r="S1" s="98"/>
+      <c r="T1" s="98"/>
+      <c r="U1" s="98"/>
+      <c r="V1" s="98"/>
+      <c r="W1" s="98"/>
+      <c r="X1" s="99"/>
+      <c r="AA1" s="117" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB1" s="118"/>
+      <c r="AC1" s="118"/>
+      <c r="AD1" s="119"/>
+    </row>
+    <row r="2" spans="1:30" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="100" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="69"/>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69"/>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="69"/>
-      <c r="S2" s="69"/>
-      <c r="T2" s="69"/>
-      <c r="U2" s="69"/>
-      <c r="V2" s="69"/>
-      <c r="W2" s="69"/>
-      <c r="X2" s="70"/>
-    </row>
-    <row r="3" spans="1:24" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="63" t="s">
+      <c r="B2" s="101"/>
+      <c r="C2" s="101"/>
+      <c r="D2" s="101"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="101"/>
+      <c r="H2" s="101"/>
+      <c r="I2" s="101"/>
+      <c r="J2" s="101"/>
+      <c r="K2" s="101"/>
+      <c r="L2" s="101"/>
+      <c r="M2" s="101"/>
+      <c r="N2" s="101"/>
+      <c r="O2" s="101"/>
+      <c r="P2" s="101"/>
+      <c r="Q2" s="101"/>
+      <c r="R2" s="101"/>
+      <c r="S2" s="101"/>
+      <c r="T2" s="101"/>
+      <c r="U2" s="101"/>
+      <c r="V2" s="101"/>
+      <c r="W2" s="101"/>
+      <c r="X2" s="102"/>
+      <c r="AA2" s="120" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB2" s="122"/>
+      <c r="AC2" s="122"/>
+      <c r="AD2" s="123"/>
+    </row>
+    <row r="3" spans="1:30" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="47" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="64" t="s">
+      <c r="C3" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="65" t="s">
+      <c r="D3" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="66" t="s">
+      <c r="E3" s="52" t="s">
         <v>82</v>
       </c>
-      <c r="F3" s="67" t="s">
+      <c r="F3" s="53" t="s">
         <v>83</v>
       </c>
-      <c r="G3" s="59"/>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="G3" s="45"/>
+      <c r="AA3" s="124"/>
+      <c r="AB3" s="125"/>
+      <c r="AC3" s="125"/>
+      <c r="AD3" s="126"/>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>1</v>
       </c>
-      <c r="B4" s="77" t="s">
+      <c r="B4" s="60" t="s">
         <v>85</v>
       </c>
       <c r="C4" s="7" t="s">
@@ -1619,18 +1916,22 @@
       <c r="D4" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="71">
+      <c r="E4" s="54">
         <v>201</v>
       </c>
-      <c r="F4" s="72">
+      <c r="F4" s="55">
         <v>201</v>
       </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="AA4" s="124"/>
+      <c r="AB4" s="125"/>
+      <c r="AC4" s="125"/>
+      <c r="AD4" s="126"/>
+    </row>
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="B5" s="78" t="s">
+      <c r="B5" s="63" t="s">
         <v>86</v>
       </c>
       <c r="C5" s="9" t="s">
@@ -1642,15 +1943,19 @@
       <c r="E5" s="24">
         <v>200</v>
       </c>
-      <c r="F5" s="73">
+      <c r="F5" s="56">
         <v>200</v>
       </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="AA5" s="124"/>
+      <c r="AB5" s="125"/>
+      <c r="AC5" s="125"/>
+      <c r="AD5" s="126"/>
+    </row>
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>3</v>
       </c>
-      <c r="B6" s="79" t="s">
+      <c r="B6" s="62" t="s">
         <v>87</v>
       </c>
       <c r="C6" s="9" t="s">
@@ -1662,15 +1967,19 @@
       <c r="E6" s="24">
         <v>200</v>
       </c>
-      <c r="F6" s="73">
+      <c r="F6" s="56">
         <v>200</v>
       </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="AA6" s="124"/>
+      <c r="AB6" s="125"/>
+      <c r="AC6" s="125"/>
+      <c r="AD6" s="126"/>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>4</v>
       </c>
-      <c r="B7" s="80" t="s">
+      <c r="B7" s="63" t="s">
         <v>88</v>
       </c>
       <c r="C7" s="9" t="s">
@@ -1682,15 +1991,19 @@
       <c r="E7" s="24">
         <v>200</v>
       </c>
-      <c r="F7" s="73">
+      <c r="F7" s="56">
         <v>200</v>
       </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="AA7" s="124"/>
+      <c r="AB7" s="125"/>
+      <c r="AC7" s="125"/>
+      <c r="AD7" s="126"/>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>5</v>
       </c>
-      <c r="B8" s="79" t="s">
+      <c r="B8" s="62" t="s">
         <v>88</v>
       </c>
       <c r="C8" s="9" t="s">
@@ -1702,15 +2015,19 @@
       <c r="E8" s="24">
         <v>200</v>
       </c>
-      <c r="F8" s="73">
+      <c r="F8" s="56">
         <v>200</v>
       </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="AA8" s="124"/>
+      <c r="AB8" s="125"/>
+      <c r="AC8" s="125"/>
+      <c r="AD8" s="126"/>
+    </row>
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>6</v>
       </c>
-      <c r="B9" s="78" t="s">
+      <c r="B9" s="61" t="s">
         <v>88</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -1722,59 +2039,71 @@
       <c r="E9" s="24">
         <v>201</v>
       </c>
-      <c r="F9" s="73">
+      <c r="F9" s="56">
         <v>201</v>
       </c>
-    </row>
-    <row r="10" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="AA9" s="124"/>
+      <c r="AB9" s="125"/>
+      <c r="AC9" s="125"/>
+      <c r="AD9" s="126"/>
+    </row>
+    <row r="10" spans="1:30" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10">
         <v>7</v>
       </c>
-      <c r="B10" s="81" t="s">
+      <c r="B10" s="64" t="s">
         <v>88</v>
       </c>
-      <c r="C10" s="62" t="s">
+      <c r="C10" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="76" t="s">
+      <c r="D10" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="74">
+      <c r="E10" s="57">
         <v>404</v>
       </c>
-      <c r="F10" s="75">
+      <c r="F10" s="58">
         <v>404</v>
       </c>
-    </row>
-    <row r="11" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="50" t="s">
+      <c r="AA10" s="124"/>
+      <c r="AB10" s="125"/>
+      <c r="AC10" s="125"/>
+      <c r="AD10" s="126"/>
+    </row>
+    <row r="11" spans="1:30" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A11" s="103" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="51"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
-      <c r="E11" s="51"/>
-      <c r="F11" s="51"/>
-      <c r="G11" s="51"/>
-      <c r="H11" s="51"/>
-      <c r="I11" s="51"/>
-      <c r="J11" s="51"/>
-      <c r="K11" s="51"/>
-      <c r="L11" s="51"/>
-      <c r="M11" s="51"/>
-      <c r="N11" s="51"/>
-      <c r="O11" s="51"/>
-      <c r="P11" s="51"/>
-      <c r="Q11" s="51"/>
-      <c r="R11" s="51"/>
-      <c r="S11" s="51"/>
-      <c r="T11" s="51"/>
-      <c r="U11" s="51"/>
-      <c r="V11" s="51"/>
-      <c r="W11" s="51"/>
-      <c r="X11" s="52"/>
-    </row>
-    <row r="12" spans="1:24" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="95"/>
+      <c r="C11" s="95"/>
+      <c r="D11" s="95"/>
+      <c r="E11" s="95"/>
+      <c r="F11" s="95"/>
+      <c r="G11" s="95"/>
+      <c r="H11" s="95"/>
+      <c r="I11" s="95"/>
+      <c r="J11" s="95"/>
+      <c r="K11" s="95"/>
+      <c r="L11" s="95"/>
+      <c r="M11" s="95"/>
+      <c r="N11" s="95"/>
+      <c r="O11" s="95"/>
+      <c r="P11" s="95"/>
+      <c r="Q11" s="95"/>
+      <c r="R11" s="95"/>
+      <c r="S11" s="95"/>
+      <c r="T11" s="95"/>
+      <c r="U11" s="95"/>
+      <c r="V11" s="95"/>
+      <c r="W11" s="95"/>
+      <c r="X11" s="96"/>
+      <c r="AA11" s="127"/>
+      <c r="AB11" s="128"/>
+      <c r="AC11" s="128"/>
+      <c r="AD11" s="129"/>
+    </row>
+    <row r="12" spans="1:30" ht="28.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="16" t="s">
         <v>13</v>
@@ -1782,7 +2111,7 @@
       <c r="C12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="58" t="s">
+      <c r="D12" s="44" t="s">
         <v>82</v>
       </c>
       <c r="E12" s="12" t="s">
@@ -1792,7 +2121,9 @@
         <v>39</v>
       </c>
       <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
+      <c r="H12" s="130" t="s">
+        <v>112</v>
+      </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
@@ -1809,9 +2140,13 @@
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
       <c r="X12" s="1"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A13" s="53" t="s">
+      <c r="AA12" s="121"/>
+      <c r="AB12" s="121"/>
+      <c r="AC12" s="121"/>
+      <c r="AD12" s="121"/>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="A13" s="104" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="15" t="s">
@@ -1846,8 +2181,8 @@
       <c r="W13" s="1"/>
       <c r="X13" s="1"/>
     </row>
-    <row r="14" spans="1:24" ht="28.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="54"/>
+    <row r="14" spans="1:30" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="105"/>
       <c r="B14" s="13" t="s">
         <v>20</v>
       </c>
@@ -1882,8 +2217,8 @@
       <c r="W14" s="1"/>
       <c r="X14" s="1"/>
     </row>
-    <row r="15" spans="1:24" ht="28.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="54"/>
+    <row r="15" spans="1:30" ht="28.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="105"/>
       <c r="B15" s="13" t="s">
         <v>21</v>
       </c>
@@ -1918,8 +2253,8 @@
       <c r="W15" s="1"/>
       <c r="X15" s="1"/>
     </row>
-    <row r="16" spans="1:24" ht="42" x14ac:dyDescent="0.3">
-      <c r="A16" s="54"/>
+    <row r="16" spans="1:30" ht="42" x14ac:dyDescent="0.3">
+      <c r="A16" s="105"/>
       <c r="B16" s="13" t="s">
         <v>25</v>
       </c>
@@ -1955,7 +2290,7 @@
       <c r="X16" s="1"/>
     </row>
     <row r="17" spans="1:24" ht="42" x14ac:dyDescent="0.3">
-      <c r="A17" s="54"/>
+      <c r="A17" s="105"/>
       <c r="B17" s="14" t="s">
         <v>26</v>
       </c>
@@ -1991,7 +2326,7 @@
       <c r="X17" s="1"/>
     </row>
     <row r="18" spans="1:24" ht="42" x14ac:dyDescent="0.3">
-      <c r="A18" s="54"/>
+      <c r="A18" s="105"/>
       <c r="B18" s="13" t="s">
         <v>28</v>
       </c>
@@ -2009,7 +2344,7 @@
       </c>
     </row>
     <row r="19" spans="1:24" ht="28.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="54"/>
+      <c r="A19" s="105"/>
       <c r="B19" s="14" t="s">
         <v>32</v>
       </c>
@@ -2027,7 +2362,7 @@
       </c>
     </row>
     <row r="20" spans="1:24" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="54"/>
+      <c r="A20" s="105"/>
       <c r="B20" s="13" t="s">
         <v>34</v>
       </c>
@@ -2045,7 +2380,7 @@
       </c>
     </row>
     <row r="21" spans="1:24" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="55"/>
+      <c r="A21" s="106"/>
       <c r="B21" s="29" t="s">
         <v>36</v>
       </c>
@@ -2063,34 +2398,34 @@
       </c>
     </row>
     <row r="22" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A22" s="56" t="s">
+      <c r="A22" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="57"/>
-      <c r="C22" s="57"/>
-      <c r="D22" s="57"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="51"/>
-      <c r="H22" s="51"/>
-      <c r="I22" s="51"/>
-      <c r="J22" s="51"/>
-      <c r="K22" s="51"/>
-      <c r="L22" s="51"/>
-      <c r="M22" s="51"/>
-      <c r="N22" s="51"/>
-      <c r="O22" s="51"/>
-      <c r="P22" s="51"/>
-      <c r="Q22" s="51"/>
-      <c r="R22" s="51"/>
-      <c r="S22" s="51"/>
-      <c r="T22" s="51"/>
-      <c r="U22" s="51"/>
-      <c r="V22" s="51"/>
-      <c r="W22" s="51"/>
-      <c r="X22" s="52"/>
-    </row>
-    <row r="23" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="94"/>
+      <c r="C22" s="94"/>
+      <c r="D22" s="94"/>
+      <c r="E22" s="94"/>
+      <c r="F22" s="94"/>
+      <c r="G22" s="95"/>
+      <c r="H22" s="95"/>
+      <c r="I22" s="95"/>
+      <c r="J22" s="95"/>
+      <c r="K22" s="95"/>
+      <c r="L22" s="95"/>
+      <c r="M22" s="95"/>
+      <c r="N22" s="95"/>
+      <c r="O22" s="95"/>
+      <c r="P22" s="95"/>
+      <c r="Q22" s="95"/>
+      <c r="R22" s="95"/>
+      <c r="S22" s="95"/>
+      <c r="T22" s="95"/>
+      <c r="U22" s="95"/>
+      <c r="V22" s="95"/>
+      <c r="W22" s="95"/>
+      <c r="X22" s="96"/>
+    </row>
+    <row r="23" spans="1:24" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="4" t="s">
         <v>13</v>
@@ -2108,7 +2443,9 @@
         <v>39</v>
       </c>
       <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
+      <c r="H23" s="130" t="s">
+        <v>112</v>
+      </c>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
@@ -2127,7 +2464,7 @@
       <c r="X23" s="1"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="111" t="s">
         <v>17</v>
       </c>
       <c r="B24" s="15" t="s">
@@ -2163,7 +2500,7 @@
       <c r="X24" s="1"/>
     </row>
     <row r="25" spans="1:24" ht="28.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="45"/>
+      <c r="A25" s="112"/>
       <c r="B25" s="13" t="s">
         <v>48</v>
       </c>
@@ -2199,7 +2536,7 @@
       <c r="X25" s="1"/>
     </row>
     <row r="26" spans="1:24" ht="42" x14ac:dyDescent="0.3">
-      <c r="A26" s="45"/>
+      <c r="A26" s="112"/>
       <c r="B26" s="13" t="s">
         <v>20</v>
       </c>
@@ -2235,7 +2572,7 @@
       <c r="X26" s="1"/>
     </row>
     <row r="27" spans="1:24" ht="42" x14ac:dyDescent="0.3">
-      <c r="A27" s="45"/>
+      <c r="A27" s="112"/>
       <c r="B27" s="13" t="s">
         <v>49</v>
       </c>
@@ -2271,7 +2608,7 @@
       <c r="X27" s="1"/>
     </row>
     <row r="28" spans="1:24" ht="69.599999999999994" x14ac:dyDescent="0.3">
-      <c r="A28" s="45"/>
+      <c r="A28" s="112"/>
       <c r="B28" s="14" t="s">
         <v>36</v>
       </c>
@@ -2307,7 +2644,7 @@
       <c r="X28" s="1"/>
     </row>
     <row r="29" spans="1:24" ht="42" x14ac:dyDescent="0.3">
-      <c r="A29" s="45"/>
+      <c r="A29" s="112"/>
       <c r="B29" s="13" t="s">
         <v>50</v>
       </c>
@@ -2325,7 +2662,7 @@
       </c>
     </row>
     <row r="30" spans="1:24" ht="55.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="45"/>
+      <c r="A30" s="112"/>
       <c r="B30" s="14" t="s">
         <v>51</v>
       </c>
@@ -2343,7 +2680,7 @@
       </c>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A31" s="45"/>
+      <c r="A31" s="112"/>
       <c r="B31" s="13" t="s">
         <v>52</v>
       </c>
@@ -2361,7 +2698,7 @@
       </c>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A32" s="45"/>
+      <c r="A32" s="112"/>
       <c r="B32" s="14" t="s">
         <v>53</v>
       </c>
@@ -2379,7 +2716,7 @@
       </c>
     </row>
     <row r="33" spans="1:24" ht="55.8" x14ac:dyDescent="0.3">
-      <c r="A33" s="45"/>
+      <c r="A33" s="112"/>
       <c r="B33" s="13" t="s">
         <v>54</v>
       </c>
@@ -2397,7 +2734,7 @@
       </c>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A34" s="45"/>
+      <c r="A34" s="112"/>
       <c r="B34" s="14" t="s">
         <v>56</v>
       </c>
@@ -2407,13 +2744,13 @@
       <c r="D34" s="23">
         <v>200</v>
       </c>
-      <c r="E34" s="84" t="s">
+      <c r="E34" s="67" t="s">
         <v>38</v>
       </c>
       <c r="F34" s="38"/>
     </row>
     <row r="35" spans="1:24" ht="69" x14ac:dyDescent="0.3">
-      <c r="A35" s="45"/>
+      <c r="A35" s="112"/>
       <c r="B35" s="13" t="s">
         <v>55</v>
       </c>
@@ -2431,7 +2768,7 @@
       </c>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A36" s="45"/>
+      <c r="A36" s="112"/>
       <c r="B36" s="14" t="s">
         <v>57</v>
       </c>
@@ -2441,13 +2778,13 @@
       <c r="D36" s="23">
         <v>200</v>
       </c>
-      <c r="E36" s="84" t="s">
+      <c r="E36" s="67" t="s">
         <v>38</v>
       </c>
       <c r="F36" s="38"/>
     </row>
     <row r="37" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="46"/>
+      <c r="A37" s="113"/>
       <c r="B37" s="40" t="s">
         <v>58</v>
       </c>
@@ -2463,45 +2800,45 @@
       <c r="F37" s="43"/>
     </row>
     <row r="38" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A38" s="56" t="s">
+      <c r="A38" s="103" t="s">
         <v>89</v>
       </c>
-      <c r="B38" s="57"/>
-      <c r="C38" s="57"/>
-      <c r="D38" s="57"/>
-      <c r="E38" s="57"/>
-      <c r="F38" s="57"/>
-      <c r="G38" s="57"/>
-      <c r="H38" s="57"/>
-      <c r="I38" s="51"/>
-      <c r="J38" s="51"/>
-      <c r="K38" s="51"/>
-      <c r="L38" s="51"/>
-      <c r="M38" s="51"/>
-      <c r="N38" s="51"/>
-      <c r="O38" s="51"/>
-      <c r="P38" s="51"/>
-      <c r="Q38" s="51"/>
-      <c r="R38" s="51"/>
-      <c r="S38" s="51"/>
-      <c r="T38" s="51"/>
-      <c r="U38" s="51"/>
-      <c r="V38" s="51"/>
-      <c r="W38" s="51"/>
-      <c r="X38" s="52"/>
+      <c r="B38" s="95"/>
+      <c r="C38" s="95"/>
+      <c r="D38" s="95"/>
+      <c r="E38" s="95"/>
+      <c r="F38" s="95"/>
+      <c r="G38" s="95"/>
+      <c r="H38" s="95"/>
+      <c r="I38" s="95"/>
+      <c r="J38" s="95"/>
+      <c r="K38" s="95"/>
+      <c r="L38" s="95"/>
+      <c r="M38" s="95"/>
+      <c r="N38" s="95"/>
+      <c r="O38" s="95"/>
+      <c r="P38" s="95"/>
+      <c r="Q38" s="95"/>
+      <c r="R38" s="95"/>
+      <c r="S38" s="95"/>
+      <c r="T38" s="95"/>
+      <c r="U38" s="95"/>
+      <c r="V38" s="95"/>
+      <c r="W38" s="95"/>
+      <c r="X38" s="96"/>
     </row>
     <row r="39" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="3"/>
       <c r="B39" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C39" s="91" t="s">
+      <c r="C39" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="D39" s="92" t="s">
+      <c r="D39" s="75" t="s">
         <v>90</v>
       </c>
-      <c r="E39" s="85" t="s">
+      <c r="E39" s="68" t="s">
         <v>22</v>
       </c>
       <c r="F39" s="35" t="s">
@@ -2515,112 +2852,112 @@
       </c>
     </row>
     <row r="40" spans="1:24" ht="54.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="44" t="s">
+      <c r="A40" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="B40" s="98" t="s">
+      <c r="B40" s="81" t="s">
         <v>91</v>
       </c>
-      <c r="C40" s="96" t="s">
+      <c r="C40" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="D40" s="99" t="s">
+      <c r="D40" s="82" t="s">
         <v>87</v>
       </c>
-      <c r="E40" s="100" t="s">
+      <c r="E40" s="83" t="s">
         <v>92</v>
       </c>
-      <c r="F40" s="101">
+      <c r="F40" s="84">
         <v>200</v>
       </c>
-      <c r="G40" s="102" t="s">
+      <c r="G40" s="85" t="s">
         <v>38</v>
       </c>
-      <c r="H40" s="103" t="s">
+      <c r="H40" s="86" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A41" s="45"/>
-      <c r="B41" s="104" t="s">
+      <c r="A41" s="105"/>
+      <c r="B41" s="87" t="s">
         <v>96</v>
       </c>
-      <c r="C41" s="90" t="s">
+      <c r="C41" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="D41" s="95" t="s">
+      <c r="D41" s="107" t="s">
         <v>88</v>
       </c>
-      <c r="E41" s="86" t="s">
+      <c r="E41" s="69" t="s">
         <v>97</v>
       </c>
       <c r="F41" s="23">
         <v>403</v>
       </c>
-      <c r="G41" s="84" t="s">
+      <c r="G41" s="67" t="s">
         <v>38</v>
       </c>
       <c r="H41" s="27"/>
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A42" s="45"/>
-      <c r="B42" s="104" t="s">
+      <c r="A42" s="105"/>
+      <c r="B42" s="87" t="s">
         <v>95</v>
       </c>
-      <c r="C42" s="90" t="s">
+      <c r="C42" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="D42" s="95" t="s">
+      <c r="D42" s="78" t="s">
         <v>88</v>
       </c>
-      <c r="E42" s="86" t="s">
+      <c r="E42" s="69" t="s">
         <v>97</v>
       </c>
       <c r="F42" s="23">
         <v>403</v>
       </c>
-      <c r="G42" s="84" t="s">
+      <c r="G42" s="67" t="s">
         <v>38</v>
       </c>
       <c r="H42" s="27"/>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A43" s="45"/>
-      <c r="B43" s="104" t="s">
+      <c r="A43" s="105"/>
+      <c r="B43" s="87" t="s">
         <v>94</v>
       </c>
-      <c r="C43" s="90" t="s">
+      <c r="C43" s="73" t="s">
         <v>11</v>
       </c>
-      <c r="D43" s="95" t="s">
+      <c r="D43" s="78" t="s">
         <v>88</v>
       </c>
-      <c r="E43" s="86" t="s">
+      <c r="E43" s="69" t="s">
         <v>97</v>
       </c>
       <c r="F43" s="23">
         <v>403</v>
       </c>
-      <c r="G43" s="84" t="s">
+      <c r="G43" s="67" t="s">
         <v>38</v>
       </c>
       <c r="H43" s="27"/>
     </row>
     <row r="44" spans="1:24" ht="42" x14ac:dyDescent="0.3">
-      <c r="A44" s="45"/>
-      <c r="B44" s="105" t="s">
+      <c r="A44" s="105"/>
+      <c r="B44" s="88" t="s">
         <v>103</v>
       </c>
-      <c r="C44" s="90" t="s">
+      <c r="C44" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="D44" s="97" t="s">
+      <c r="D44" s="80" t="s">
         <v>86</v>
       </c>
-      <c r="E44" s="109" t="s">
+      <c r="E44" s="92" t="s">
         <v>104</v>
       </c>
-      <c r="F44" s="108">
+      <c r="F44" s="91">
         <v>401</v>
       </c>
       <c r="G44" s="25" t="s">
@@ -2631,17 +2968,17 @@
       </c>
     </row>
     <row r="45" spans="1:24" ht="42" x14ac:dyDescent="0.3">
-      <c r="A45" s="45"/>
-      <c r="B45" s="106" t="s">
+      <c r="A45" s="105"/>
+      <c r="B45" s="89" t="s">
         <v>100</v>
       </c>
-      <c r="C45" s="90" t="s">
+      <c r="C45" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="D45" s="97" t="s">
+      <c r="D45" s="80" t="s">
         <v>86</v>
       </c>
-      <c r="E45" s="88" t="s">
+      <c r="E45" s="71" t="s">
         <v>98</v>
       </c>
       <c r="F45" s="23">
@@ -2655,17 +2992,17 @@
       </c>
     </row>
     <row r="46" spans="1:24" ht="55.2" x14ac:dyDescent="0.3">
-      <c r="A46" s="45"/>
-      <c r="B46" s="106" t="s">
+      <c r="A46" s="105"/>
+      <c r="B46" s="89" t="s">
         <v>101</v>
       </c>
-      <c r="C46" s="90" t="s">
+      <c r="C46" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="D46" s="97" t="s">
+      <c r="D46" s="80" t="s">
         <v>86</v>
       </c>
-      <c r="E46" s="88" t="s">
+      <c r="E46" s="71" t="s">
         <v>102</v>
       </c>
       <c r="F46" s="23">
@@ -2679,80 +3016,934 @@
       </c>
     </row>
     <row r="47" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A47" s="45"/>
-      <c r="B47" s="104"/>
-      <c r="C47" s="90"/>
-      <c r="D47" s="60"/>
-      <c r="E47" s="87"/>
+      <c r="A47" s="105"/>
+      <c r="B47" s="87"/>
+      <c r="C47" s="73"/>
+      <c r="D47" s="46"/>
+      <c r="E47" s="70"/>
       <c r="F47" s="23"/>
-      <c r="G47" s="83"/>
+      <c r="G47" s="66"/>
       <c r="H47" s="27"/>
     </row>
     <row r="48" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A48" s="45"/>
-      <c r="B48" s="106"/>
-      <c r="C48" s="90"/>
-      <c r="D48" s="60"/>
-      <c r="E48" s="87"/>
+      <c r="A48" s="105"/>
+      <c r="B48" s="89"/>
+      <c r="C48" s="73"/>
+      <c r="D48" s="46"/>
+      <c r="E48" s="70"/>
       <c r="F48" s="23"/>
-      <c r="G48" s="83"/>
+      <c r="G48" s="66"/>
       <c r="H48" s="27"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A49" s="45"/>
-      <c r="B49" s="104"/>
-      <c r="C49" s="90"/>
-      <c r="D49" s="60"/>
-      <c r="E49" s="87"/>
+    <row r="49" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A49" s="105"/>
+      <c r="B49" s="87"/>
+      <c r="C49" s="73"/>
+      <c r="D49" s="46"/>
+      <c r="E49" s="70"/>
       <c r="F49" s="23"/>
-      <c r="G49" s="83"/>
+      <c r="G49" s="66"/>
       <c r="H49" s="27"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A50" s="45"/>
-      <c r="B50" s="106"/>
-      <c r="C50" s="90"/>
-      <c r="D50" s="60"/>
-      <c r="E50" s="87"/>
+    <row r="50" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A50" s="105"/>
+      <c r="B50" s="89"/>
+      <c r="C50" s="73"/>
+      <c r="D50" s="46"/>
+      <c r="E50" s="70"/>
       <c r="F50" s="23"/>
-      <c r="G50" s="83"/>
+      <c r="G50" s="66"/>
       <c r="H50" s="38"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A51" s="45"/>
-      <c r="B51" s="104"/>
-      <c r="C51" s="90"/>
-      <c r="D51" s="60"/>
+    <row r="51" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A51" s="105"/>
+      <c r="B51" s="87"/>
+      <c r="C51" s="73"/>
+      <c r="D51" s="46"/>
       <c r="E51" s="39"/>
       <c r="F51" s="23"/>
-      <c r="G51" s="83"/>
+      <c r="G51" s="66"/>
       <c r="H51" s="27"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A52" s="45"/>
-      <c r="B52" s="106"/>
-      <c r="C52" s="90"/>
-      <c r="D52" s="60"/>
-      <c r="E52" s="87"/>
+    <row r="52" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A52" s="105"/>
+      <c r="B52" s="89"/>
+      <c r="C52" s="73"/>
+      <c r="D52" s="46"/>
+      <c r="E52" s="70"/>
       <c r="F52" s="23"/>
-      <c r="G52" s="83"/>
+      <c r="G52" s="66"/>
       <c r="H52" s="38"/>
     </row>
-    <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="46"/>
-      <c r="B53" s="107"/>
-      <c r="C53" s="93"/>
-      <c r="D53" s="94"/>
-      <c r="E53" s="89"/>
+    <row r="53" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="106"/>
+      <c r="B53" s="90"/>
+      <c r="C53" s="76"/>
+      <c r="D53" s="77"/>
+      <c r="E53" s="72"/>
       <c r="F53" s="41"/>
-      <c r="G53" s="82"/>
+      <c r="G53" s="65"/>
       <c r="H53" s="43"/>
     </row>
+    <row r="54" spans="1:25" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A54" s="103" t="s">
+        <v>105</v>
+      </c>
+      <c r="B54" s="95"/>
+      <c r="C54" s="95"/>
+      <c r="D54" s="95"/>
+      <c r="E54" s="95"/>
+      <c r="F54" s="95"/>
+      <c r="G54" s="95"/>
+      <c r="H54" s="95"/>
+      <c r="I54" s="95"/>
+      <c r="J54" s="95"/>
+      <c r="K54" s="95"/>
+      <c r="L54" s="95"/>
+      <c r="M54" s="95"/>
+      <c r="N54" s="95"/>
+      <c r="O54" s="95"/>
+      <c r="P54" s="95"/>
+      <c r="Q54" s="95"/>
+      <c r="R54" s="95"/>
+      <c r="S54" s="95"/>
+      <c r="T54" s="95"/>
+      <c r="U54" s="95"/>
+      <c r="V54" s="95"/>
+      <c r="W54" s="95"/>
+      <c r="X54" s="96"/>
+    </row>
+    <row r="55" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B55" s="1"/>
+      <c r="C55" s="139"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
+      <c r="I55" s="1"/>
+      <c r="J55" s="1"/>
+      <c r="K55" s="1"/>
+      <c r="L55" s="1"/>
+      <c r="M55" s="1"/>
+      <c r="N55" s="1"/>
+      <c r="O55" s="1"/>
+      <c r="P55" s="1"/>
+      <c r="Q55" s="1"/>
+      <c r="R55" s="1"/>
+      <c r="S55" s="1"/>
+      <c r="T55" s="1"/>
+      <c r="U55" s="1"/>
+      <c r="V55" s="1"/>
+      <c r="W55" s="1"/>
+      <c r="X55" s="1"/>
+    </row>
+    <row r="56" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="3"/>
+      <c r="B56" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C56" s="140" t="s">
+        <v>14</v>
+      </c>
+      <c r="D56" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="E56" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="F56" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="G56" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H56" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I56" s="1"/>
+      <c r="J56" s="1"/>
+      <c r="K56" s="1"/>
+      <c r="L56" s="1"/>
+      <c r="M56" s="1"/>
+      <c r="N56" s="1"/>
+      <c r="O56" s="1"/>
+      <c r="P56" s="1"/>
+      <c r="Q56" s="1"/>
+      <c r="R56" s="1"/>
+      <c r="S56" s="1"/>
+      <c r="T56" s="1"/>
+      <c r="U56" s="1"/>
+      <c r="V56" s="1"/>
+      <c r="W56" s="1"/>
+      <c r="X56" s="1"/>
+    </row>
+    <row r="57" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A57" s="104" t="s">
+        <v>17</v>
+      </c>
+      <c r="B57" s="81" t="s">
+        <v>2</v>
+      </c>
+      <c r="C57" s="148" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" s="149" t="s">
+        <v>86</v>
+      </c>
+      <c r="E57" s="83" t="s">
+        <v>109</v>
+      </c>
+      <c r="F57" s="84">
+        <v>200</v>
+      </c>
+      <c r="G57" s="85" t="s">
+        <v>38</v>
+      </c>
+      <c r="H57" s="114"/>
+      <c r="I57" s="1"/>
+      <c r="J57" s="1"/>
+      <c r="K57" s="1"/>
+      <c r="L57" s="1"/>
+      <c r="M57" s="1"/>
+      <c r="N57" s="1"/>
+      <c r="O57" s="1"/>
+      <c r="P57" s="1"/>
+      <c r="Q57" s="1"/>
+      <c r="R57" s="1"/>
+      <c r="S57" s="1"/>
+      <c r="T57" s="1"/>
+      <c r="U57" s="1"/>
+      <c r="V57" s="1"/>
+      <c r="W57" s="1"/>
+      <c r="X57" s="1"/>
+    </row>
+    <row r="58" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A58" s="105"/>
+      <c r="B58" s="87" t="s">
+        <v>3</v>
+      </c>
+      <c r="C58" s="143" t="s">
+        <v>9</v>
+      </c>
+      <c r="D58" s="150" t="s">
+        <v>87</v>
+      </c>
+      <c r="E58" s="69" t="s">
+        <v>97</v>
+      </c>
+      <c r="F58" s="23">
+        <v>200</v>
+      </c>
+      <c r="G58" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H58" s="115"/>
+      <c r="I58" s="1"/>
+      <c r="J58" s="1"/>
+      <c r="K58" s="1"/>
+      <c r="L58" s="1"/>
+      <c r="M58" s="1"/>
+      <c r="N58" s="1"/>
+      <c r="O58" s="1"/>
+      <c r="P58" s="1"/>
+      <c r="Q58" s="1"/>
+      <c r="R58" s="1"/>
+      <c r="S58" s="1"/>
+      <c r="T58" s="1"/>
+      <c r="U58" s="1"/>
+      <c r="V58" s="1"/>
+      <c r="W58" s="1"/>
+      <c r="X58" s="1"/>
+    </row>
+    <row r="59" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A59" s="105"/>
+      <c r="B59" s="87" t="s">
+        <v>106</v>
+      </c>
+      <c r="C59" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" s="150" t="s">
+        <v>108</v>
+      </c>
+      <c r="E59" s="69" t="s">
+        <v>110</v>
+      </c>
+      <c r="F59" s="23">
+        <v>200</v>
+      </c>
+      <c r="G59" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H59" s="115"/>
+      <c r="I59" s="1"/>
+      <c r="J59" s="1"/>
+      <c r="K59" s="1"/>
+      <c r="L59" s="1"/>
+      <c r="M59" s="1"/>
+      <c r="N59" s="1"/>
+      <c r="O59" s="1"/>
+      <c r="P59" s="1"/>
+      <c r="Q59" s="1"/>
+      <c r="R59" s="1"/>
+      <c r="S59" s="1"/>
+      <c r="T59" s="1"/>
+      <c r="U59" s="1"/>
+      <c r="V59" s="1"/>
+      <c r="W59" s="1"/>
+      <c r="X59" s="1"/>
+    </row>
+    <row r="60" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A60" s="105"/>
+      <c r="B60" s="87" t="s">
+        <v>107</v>
+      </c>
+      <c r="C60" s="143" t="s">
+        <v>11</v>
+      </c>
+      <c r="D60" s="151" t="s">
+        <v>88</v>
+      </c>
+      <c r="E60" s="69" t="s">
+        <v>111</v>
+      </c>
+      <c r="F60" s="23">
+        <v>200</v>
+      </c>
+      <c r="G60" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H60" s="115"/>
+      <c r="I60" s="131"/>
+      <c r="J60" s="132"/>
+      <c r="K60" s="132"/>
+      <c r="L60" s="132"/>
+      <c r="M60" s="132"/>
+      <c r="N60" s="132"/>
+      <c r="O60" s="132"/>
+      <c r="P60" s="132"/>
+      <c r="Q60" s="132"/>
+      <c r="R60" s="132"/>
+      <c r="S60" s="132"/>
+      <c r="T60" s="132"/>
+      <c r="U60" s="132"/>
+      <c r="V60" s="132"/>
+      <c r="W60" s="132"/>
+      <c r="X60" s="132"/>
+    </row>
+    <row r="61" spans="1:25" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A61" s="105"/>
+      <c r="B61" s="88" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" s="153" t="s">
+        <v>81</v>
+      </c>
+      <c r="D61" s="151" t="s">
+        <v>88</v>
+      </c>
+      <c r="E61" s="154" t="s">
+        <v>110</v>
+      </c>
+      <c r="F61" s="91">
+        <v>201</v>
+      </c>
+      <c r="G61" s="134" t="s">
+        <v>38</v>
+      </c>
+      <c r="H61" s="115"/>
+      <c r="I61" s="133"/>
+      <c r="J61" s="133"/>
+      <c r="K61" s="133"/>
+      <c r="L61" s="133"/>
+      <c r="M61" s="133"/>
+      <c r="N61" s="133"/>
+      <c r="O61" s="133"/>
+      <c r="P61" s="133"/>
+      <c r="Q61" s="133"/>
+      <c r="R61" s="133"/>
+      <c r="S61" s="133"/>
+      <c r="T61" s="133"/>
+      <c r="U61" s="133"/>
+      <c r="V61" s="133"/>
+      <c r="W61" s="133"/>
+      <c r="X61" s="133"/>
+      <c r="Y61" s="108"/>
+    </row>
+    <row r="62" spans="1:25" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A62" s="103" t="s">
+        <v>115</v>
+      </c>
+      <c r="B62" s="95"/>
+      <c r="C62" s="95"/>
+      <c r="D62" s="95"/>
+      <c r="E62" s="95"/>
+      <c r="F62" s="95"/>
+      <c r="G62" s="95"/>
+      <c r="H62" s="95"/>
+      <c r="I62" s="95"/>
+      <c r="J62" s="95"/>
+      <c r="K62" s="95"/>
+      <c r="L62" s="95"/>
+      <c r="M62" s="95"/>
+      <c r="N62" s="95"/>
+      <c r="O62" s="95"/>
+      <c r="P62" s="95"/>
+      <c r="Q62" s="95"/>
+      <c r="R62" s="95"/>
+      <c r="S62" s="95"/>
+      <c r="T62" s="95"/>
+      <c r="U62" s="95"/>
+      <c r="V62" s="95"/>
+      <c r="W62" s="95"/>
+      <c r="X62" s="96"/>
+    </row>
+    <row r="63" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>125</v>
+      </c>
+      <c r="B63" s="1"/>
+      <c r="C63" s="139"/>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1"/>
+      <c r="G63" s="1"/>
+      <c r="H63" s="1"/>
+      <c r="I63" s="1"/>
+      <c r="J63" s="1"/>
+      <c r="K63" s="1"/>
+      <c r="L63" s="1"/>
+      <c r="M63" s="1"/>
+      <c r="N63" s="1"/>
+      <c r="O63" s="1"/>
+      <c r="P63" s="1"/>
+      <c r="Q63" s="1"/>
+      <c r="R63" s="1"/>
+      <c r="S63" s="1"/>
+      <c r="T63" s="1"/>
+      <c r="U63" s="1"/>
+      <c r="V63" s="1"/>
+      <c r="W63" s="1"/>
+      <c r="X63" s="1"/>
+    </row>
+    <row r="64" spans="1:25" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="3"/>
+      <c r="B64" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C64" s="140" t="s">
+        <v>14</v>
+      </c>
+      <c r="D64" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="E64" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="F64" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="G64" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H64" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I64" s="1"/>
+      <c r="J64" s="1"/>
+      <c r="K64" s="1"/>
+      <c r="L64" s="1"/>
+      <c r="M64" s="1"/>
+      <c r="N64" s="1"/>
+      <c r="O64" s="1"/>
+      <c r="P64" s="1"/>
+      <c r="Q64" s="1"/>
+      <c r="R64" s="1"/>
+      <c r="S64" s="1"/>
+      <c r="T64" s="1"/>
+      <c r="U64" s="1"/>
+      <c r="V64" s="1"/>
+      <c r="W64" s="1"/>
+      <c r="X64" s="1"/>
+    </row>
+    <row r="65" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A65" s="104" t="s">
+        <v>17</v>
+      </c>
+      <c r="B65" s="81" t="s">
+        <v>2</v>
+      </c>
+      <c r="C65" s="148" t="s">
+        <v>9</v>
+      </c>
+      <c r="D65" s="149" t="s">
+        <v>86</v>
+      </c>
+      <c r="E65" s="83" t="s">
+        <v>109</v>
+      </c>
+      <c r="F65" s="84">
+        <v>200</v>
+      </c>
+      <c r="G65" s="85" t="s">
+        <v>38</v>
+      </c>
+      <c r="H65" s="114"/>
+      <c r="I65" s="1"/>
+      <c r="J65" s="1"/>
+      <c r="K65" s="1"/>
+      <c r="L65" s="1"/>
+      <c r="M65" s="1"/>
+      <c r="N65" s="1"/>
+      <c r="O65" s="1"/>
+      <c r="P65" s="1"/>
+      <c r="Q65" s="1"/>
+      <c r="R65" s="1"/>
+      <c r="S65" s="1"/>
+      <c r="T65" s="1"/>
+      <c r="U65" s="1"/>
+      <c r="V65" s="1"/>
+      <c r="W65" s="1"/>
+      <c r="X65" s="1"/>
+    </row>
+    <row r="66" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A66" s="105"/>
+      <c r="B66" s="87" t="s">
+        <v>3</v>
+      </c>
+      <c r="C66" s="143" t="s">
+        <v>9</v>
+      </c>
+      <c r="D66" s="150" t="s">
+        <v>87</v>
+      </c>
+      <c r="E66" s="69" t="s">
+        <v>97</v>
+      </c>
+      <c r="F66" s="23">
+        <v>200</v>
+      </c>
+      <c r="G66" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H66" s="115"/>
+      <c r="I66" s="1"/>
+      <c r="J66" s="1"/>
+      <c r="K66" s="1"/>
+      <c r="L66" s="1"/>
+      <c r="M66" s="1"/>
+      <c r="N66" s="1"/>
+      <c r="O66" s="1"/>
+      <c r="P66" s="1"/>
+      <c r="Q66" s="1"/>
+      <c r="R66" s="1"/>
+      <c r="S66" s="1"/>
+      <c r="T66" s="1"/>
+      <c r="U66" s="1"/>
+      <c r="V66" s="1"/>
+      <c r="W66" s="1"/>
+      <c r="X66" s="1"/>
+    </row>
+    <row r="67" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A67" s="105"/>
+      <c r="B67" s="87" t="s">
+        <v>107</v>
+      </c>
+      <c r="C67" s="143" t="s">
+        <v>11</v>
+      </c>
+      <c r="D67" s="151" t="s">
+        <v>88</v>
+      </c>
+      <c r="E67" s="69" t="s">
+        <v>117</v>
+      </c>
+      <c r="F67" s="23">
+        <v>200</v>
+      </c>
+      <c r="G67" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H67" s="115"/>
+      <c r="I67" s="1"/>
+      <c r="J67" s="1"/>
+      <c r="K67" s="1"/>
+      <c r="L67" s="1"/>
+      <c r="M67" s="1"/>
+      <c r="N67" s="1"/>
+      <c r="O67" s="1"/>
+      <c r="P67" s="1"/>
+      <c r="Q67" s="1"/>
+      <c r="R67" s="1"/>
+      <c r="S67" s="1"/>
+      <c r="T67" s="1"/>
+      <c r="U67" s="1"/>
+      <c r="V67" s="1"/>
+      <c r="W67" s="1"/>
+      <c r="X67" s="1"/>
+    </row>
+    <row r="68" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A68" s="105"/>
+      <c r="B68" s="87" t="s">
+        <v>116</v>
+      </c>
+      <c r="C68" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="D68" s="150" t="s">
+        <v>88</v>
+      </c>
+      <c r="E68" s="69" t="s">
+        <v>110</v>
+      </c>
+      <c r="F68" s="23">
+        <v>200</v>
+      </c>
+      <c r="G68" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H68" s="115"/>
+    </row>
+    <row r="69" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="106"/>
+      <c r="B69" s="109" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" s="147" t="s">
+        <v>81</v>
+      </c>
+      <c r="D69" s="152" t="s">
+        <v>88</v>
+      </c>
+      <c r="E69" s="69" t="s">
+        <v>110</v>
+      </c>
+      <c r="F69" s="65">
+        <v>201</v>
+      </c>
+      <c r="G69" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H69" s="116"/>
+      <c r="W69" s="108"/>
+    </row>
+    <row r="70" spans="1:24" ht="25.8" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A70" s="103" t="s">
+        <v>118</v>
+      </c>
+      <c r="B70" s="95"/>
+      <c r="C70" s="95"/>
+      <c r="D70" s="95"/>
+      <c r="E70" s="95"/>
+      <c r="F70" s="95"/>
+      <c r="G70" s="95"/>
+      <c r="H70" s="95"/>
+      <c r="I70" s="95"/>
+      <c r="J70" s="95"/>
+      <c r="K70" s="95"/>
+      <c r="L70" s="95"/>
+      <c r="M70" s="95"/>
+      <c r="N70" s="95"/>
+      <c r="O70" s="95"/>
+      <c r="P70" s="95"/>
+      <c r="Q70" s="95"/>
+      <c r="R70" s="95"/>
+      <c r="S70" s="95"/>
+      <c r="T70" s="95"/>
+      <c r="U70" s="95"/>
+      <c r="V70" s="95"/>
+      <c r="W70" s="95"/>
+      <c r="X70" s="96"/>
+    </row>
+    <row r="71" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="1"/>
+      <c r="C71" s="139"/>
+      <c r="D71" s="1"/>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1"/>
+      <c r="G71" s="1"/>
+      <c r="H71" s="1"/>
+      <c r="I71" s="1"/>
+      <c r="J71" s="1"/>
+      <c r="K71" s="1"/>
+      <c r="L71" s="1"/>
+      <c r="M71" s="1"/>
+      <c r="N71" s="1"/>
+      <c r="O71" s="1"/>
+      <c r="P71" s="1"/>
+      <c r="Q71" s="1"/>
+      <c r="R71" s="1"/>
+      <c r="S71" s="1"/>
+      <c r="T71" s="1"/>
+      <c r="U71" s="1"/>
+      <c r="V71" s="1"/>
+      <c r="W71" s="1"/>
+      <c r="X71" s="1"/>
+    </row>
+    <row r="72" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="3"/>
+      <c r="B72" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C72" s="140" t="s">
+        <v>14</v>
+      </c>
+      <c r="D72" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="E72" s="68" t="s">
+        <v>22</v>
+      </c>
+      <c r="F72" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="G72" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H72" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I72" s="1"/>
+      <c r="J72" s="1"/>
+      <c r="K72" s="1"/>
+      <c r="L72" s="1"/>
+      <c r="M72" s="1"/>
+      <c r="N72" s="1"/>
+      <c r="O72" s="1"/>
+      <c r="P72" s="1"/>
+      <c r="Q72" s="1"/>
+      <c r="R72" s="1"/>
+      <c r="S72" s="1"/>
+      <c r="T72" s="1"/>
+      <c r="U72" s="1"/>
+      <c r="V72" s="1"/>
+      <c r="W72" s="1"/>
+      <c r="X72" s="1"/>
+    </row>
+    <row r="73" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A73" s="105" t="s">
+        <v>17</v>
+      </c>
+      <c r="B73" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C73" s="141" t="s">
+        <v>9</v>
+      </c>
+      <c r="D73" s="142" t="s">
+        <v>86</v>
+      </c>
+      <c r="E73" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="F73" s="22">
+        <v>200</v>
+      </c>
+      <c r="G73" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="H73" s="135"/>
+      <c r="I73" s="1"/>
+      <c r="J73" s="1"/>
+      <c r="K73" s="1"/>
+      <c r="L73" s="1"/>
+      <c r="M73" s="1"/>
+      <c r="N73" s="1"/>
+      <c r="O73" s="1"/>
+      <c r="P73" s="1"/>
+      <c r="Q73" s="1"/>
+      <c r="R73" s="1"/>
+      <c r="S73" s="1"/>
+      <c r="T73" s="1"/>
+      <c r="U73" s="1"/>
+      <c r="V73" s="1"/>
+      <c r="W73" s="1"/>
+      <c r="X73" s="1"/>
+    </row>
+    <row r="74" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A74" s="105"/>
+      <c r="B74" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C74" s="143" t="s">
+        <v>9</v>
+      </c>
+      <c r="D74" s="144" t="s">
+        <v>87</v>
+      </c>
+      <c r="E74" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="F74" s="23">
+        <v>200</v>
+      </c>
+      <c r="G74" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H74" s="27"/>
+      <c r="I74" s="1"/>
+      <c r="J74" s="1"/>
+      <c r="K74" s="1"/>
+      <c r="L74" s="1"/>
+      <c r="M74" s="1"/>
+      <c r="N74" s="1"/>
+      <c r="O74" s="1"/>
+      <c r="P74" s="1"/>
+      <c r="Q74" s="1"/>
+      <c r="R74" s="1"/>
+      <c r="S74" s="1"/>
+      <c r="T74" s="1"/>
+      <c r="U74" s="1"/>
+      <c r="V74" s="1"/>
+      <c r="W74" s="1"/>
+      <c r="X74" s="1"/>
+    </row>
+    <row r="75" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A75" s="105"/>
+      <c r="B75" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="C75" s="143" t="s">
+        <v>10</v>
+      </c>
+      <c r="D75" s="144" t="s">
+        <v>87</v>
+      </c>
+      <c r="E75" s="145" t="s">
+        <v>123</v>
+      </c>
+      <c r="F75" s="23">
+        <v>403</v>
+      </c>
+      <c r="G75" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H75" s="38"/>
+      <c r="I75" s="1"/>
+      <c r="J75" s="1"/>
+      <c r="K75" s="1"/>
+      <c r="L75" s="1"/>
+      <c r="M75" s="1"/>
+      <c r="N75" s="1"/>
+      <c r="O75" s="1"/>
+      <c r="P75" s="1"/>
+      <c r="Q75" s="1"/>
+      <c r="R75" s="1"/>
+      <c r="S75" s="1"/>
+      <c r="T75" s="1"/>
+      <c r="U75" s="1"/>
+      <c r="V75" s="1"/>
+      <c r="W75" s="1"/>
+      <c r="X75" s="1"/>
+    </row>
+    <row r="76" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A76" s="105"/>
+      <c r="B76" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C76" s="143" t="s">
+        <v>11</v>
+      </c>
+      <c r="D76" s="143" t="s">
+        <v>88</v>
+      </c>
+      <c r="E76" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="F76" s="23">
+        <v>403</v>
+      </c>
+      <c r="G76" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H76" s="27"/>
+    </row>
+    <row r="77" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A77" s="105"/>
+      <c r="B77" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="C77" s="143" t="s">
+        <v>81</v>
+      </c>
+      <c r="D77" s="143" t="s">
+        <v>88</v>
+      </c>
+      <c r="E77" s="146" t="s">
+        <v>110</v>
+      </c>
+      <c r="F77" s="66">
+        <v>403</v>
+      </c>
+      <c r="G77" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H77" s="38"/>
+      <c r="W77" s="108"/>
+    </row>
+    <row r="78" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A78" s="105"/>
+      <c r="B78" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C78" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="D78" s="144" t="s">
+        <v>88</v>
+      </c>
+      <c r="E78" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="F78" s="23">
+        <v>200</v>
+      </c>
+      <c r="G78" s="67" t="s">
+        <v>38</v>
+      </c>
+      <c r="H78" s="27"/>
+    </row>
+    <row r="79" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A79" s="106"/>
+      <c r="B79" s="40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C79" s="147" t="s">
+        <v>9</v>
+      </c>
+      <c r="D79" s="147" t="s">
+        <v>88</v>
+      </c>
+      <c r="E79" s="136" t="s">
+        <v>110</v>
+      </c>
+      <c r="F79" s="137">
+        <v>201</v>
+      </c>
+      <c r="G79" s="138" t="s">
+        <v>38</v>
+      </c>
+      <c r="H79" s="110"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="15">
+    <mergeCell ref="A65:A69"/>
+    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="A62:X62"/>
+    <mergeCell ref="A70:X70"/>
+    <mergeCell ref="A73:A79"/>
+    <mergeCell ref="AA1:AD1"/>
+    <mergeCell ref="AA2:AD11"/>
+    <mergeCell ref="A54:X54"/>
     <mergeCell ref="A38:X38"/>
     <mergeCell ref="A40:A53"/>
-    <mergeCell ref="A24:A37"/>
     <mergeCell ref="A1:X1"/>
     <mergeCell ref="A2:X2"/>
     <mergeCell ref="A11:X11"/>
@@ -2761,9 +3952,21 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B7" r:id="rId1" xr:uid="{9A88E16A-6488-4038-BE51-669306FE468A}"/>
+    <hyperlink ref="D57" r:id="rId2" xr:uid="{0BFD8C3A-1B56-4B9A-9C01-C1C60FFB4490}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{BD7070AA-29CD-4CC0-BD00-5E299118929E}"/>
+    <hyperlink ref="D58" r:id="rId4" xr:uid="{57B3ADC6-0B0A-4547-80FC-E1CAD27E2755}"/>
+    <hyperlink ref="D59" r:id="rId5" xr:uid="{74A4B992-6346-4064-A998-D77A36CAE9B1}"/>
+    <hyperlink ref="D41" r:id="rId6" xr:uid="{A24FCC40-21AA-4FB2-B0BF-55FB5E9B4451}"/>
+    <hyperlink ref="D65" r:id="rId7" xr:uid="{4C50CE3F-F7FB-41AF-AB71-3CD95A4C3475}"/>
+    <hyperlink ref="D66" r:id="rId8" xr:uid="{F33A1BB8-61D4-4A6F-A3B2-CCD91498BE2F}"/>
+    <hyperlink ref="D68" r:id="rId9" xr:uid="{C74F479E-C10F-4F6E-8DE3-BDE65614701A}"/>
+    <hyperlink ref="D73" r:id="rId10" xr:uid="{81561F4E-0B95-4A6F-842F-BDA79552BCB0}"/>
+    <hyperlink ref="D74" r:id="rId11" xr:uid="{70347EE2-6B65-43A4-B8D1-B586486FE401}"/>
+    <hyperlink ref="D78" r:id="rId12" xr:uid="{FEDA0155-D864-4B25-99F6-F6CF203C9795}"/>
+    <hyperlink ref="D75" r:id="rId13" xr:uid="{D4AA341A-A2AC-4AE7-A78D-2FDD70689BE4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId14"/>
   <ignoredErrors>
     <ignoredError sqref="C19" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>